<commit_message>
feat(data): add Urea 30/07 reagent temperature incident to Phase 2 dataset
</commit_message>
<xml_diff>
--- a/public/Bang_Du_Lieu_QC_T7_T8_2026.xlsx
+++ b/public/Bang_Du_Lieu_QC_T7_T8_2026.xlsx
@@ -1263,7 +1263,7 @@
         <v>17.38</v>
       </c>
       <c r="E23">
-        <v>7</v>
+        <v>6.45</v>
       </c>
       <c r="F23">
         <v>21.4</v>
@@ -1275,10 +1275,10 @@
         <v>347</v>
       </c>
       <c r="I23" t="str">
-        <v>Hợp lệ (In-control)</v>
+        <v>Vi phạm: UREA (Normal): Vi phạm (1-3s)</v>
       </c>
       <c r="J23" t="str">
-        <v>Không cần can thiệp</v>
+        <v>Lập biên bản CAPA theo QĐ 2429</v>
       </c>
       <c r="K23" t="str">
         <v>Đàm Minh Đức</v>

</xml_diff>